<commit_message>
data: update gym training calendar
</commit_message>
<xml_diff>
--- a/Data/GYM/gym_calendar.xlsx
+++ b/Data/GYM/gym_calendar.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
   <si>
     <t>Progress Dashboard</t>
   </si>
@@ -181,6 +181,9 @@
 Forearms:
 1. wrist curl
 2. weight squzee</t>
+  </si>
+  <si>
+    <t>is my chest day</t>
   </si>
 </sst>
 </file>
@@ -934,7 +937,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>46193</v>
       </c>
@@ -960,6 +963,9 @@
         <f>VLOOKUP(C9,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Quads, Hamstrings, Calves, Shoulders (medial+posterior delt), Core</v>
       </c>
+      <c r="F9" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -982,7 +988,7 @@
         <v>Recovery</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>46195</v>
       </c>
@@ -1007,8 +1013,11 @@
         <f>VLOOKUP(C11,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Upper Chest (priority), Triceps - long head + lateral head</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>46196</v>
       </c>
@@ -1033,8 +1042,11 @@
         <f>VLOOKUP(C12,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Lat Width, Back Thickness, Rear Delts/Posture, Biceps, Forearms</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>46197</v>
       </c>
@@ -1060,8 +1072,11 @@
         <f>VLOOKUP(C13,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Quads, Hamstrings, Calves, Shoulders (medial+posterior delt), Core</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>46198</v>
       </c>
@@ -1086,8 +1101,11 @@
         <f>VLOOKUP(C14,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Upper Chest (priority), Triceps - long head + lateral head</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>46199</v>
       </c>
@@ -1112,8 +1130,11 @@
         <f>VLOOKUP(C15,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Lat Width, Back Thickness, Rear Delts/Posture, Biceps, Forearms</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>46200</v>
       </c>
@@ -1139,6 +1160,9 @@
         <f>VLOOKUP(C16,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Quads, Hamstrings, Calves, Shoulders (medial+posterior delt), Core</v>
       </c>
+      <c r="F16" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
@@ -1161,7 +1185,7 @@
         <v>Recovery</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>46202</v>
       </c>
@@ -1186,8 +1210,11 @@
         <f>VLOOKUP(C18,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Upper Chest (priority), Triceps - long head + lateral head</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>46203</v>
       </c>
@@ -1212,8 +1239,11 @@
         <f>VLOOKUP(C19,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Lat Width, Back Thickness, Rear Delts/Posture, Biceps, Forearms</v>
       </c>
-    </row>
-    <row r="20" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" ht="14.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>46204</v>
       </c>
@@ -1239,8 +1269,11 @@
         <f>VLOOKUP(C20,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Quads, Hamstrings, Calves, Shoulders (medial+posterior delt), Core</v>
       </c>
-    </row>
-    <row r="21" ht="15.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" ht="15.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>46205</v>
       </c>
@@ -1265,8 +1298,11 @@
         <f>VLOOKUP(C21,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Upper Chest (priority), Triceps - long head + lateral head</v>
       </c>
-    </row>
-    <row r="22" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" ht="14.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>46206</v>
       </c>
@@ -1291,8 +1327,11 @@
         <f>VLOOKUP(C22,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Lat Width, Back Thickness, Rear Delts/Posture, Biceps, Forearms</v>
       </c>
-    </row>
-    <row r="23" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" ht="14.5" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>46207</v>
       </c>
@@ -1318,6 +1357,9 @@
         <f>VLOOKUP(C23,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Quads, Hamstrings, Calves, Shoulders (medial+posterior delt), Core</v>
       </c>
+      <c r="F23" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="24" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -2008,7 +2050,7 @@
         <v>Lat Width, Back Thickness, Rear Delts/Posture, Biceps, Forearms</v>
       </c>
     </row>
-    <row r="51" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" ht="14.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>46235</v>
       </c>
@@ -2034,6 +2076,12 @@
         <f>VLOOKUP(C51,'Plan (PPL Template)'!A4:C7,3,FALSE())</f>
         <v>Quads, Hamstrings, Calves, Shoulders (medial+posterior delt), Core</v>
       </c>
+      <c r="F51" t="s">
+        <v>32</v>
+      </c>
+      <c r="G51" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="52" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2">

</xml_diff>